<commit_message>
changes in edit event and schedule
</commit_message>
<xml_diff>
--- a/all requirements/participants.xlsx
+++ b/all requirements/participants.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HARDIK DHAWAN\OneDrive\Desktop\Minor project\all requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HARDIK DHAWAN\OneDrive\Desktop\Minor-Project-Food-cupons-on-events-\all requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F2F8F17-4C87-44EB-8D8A-F1D53A61C9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC942906-91A6-4B60-9167-33DF25315954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
   <si>
     <t>name</t>
   </si>
@@ -53,6 +53,12 @@
   </si>
   <si>
     <t>hardikdhawan446@gmail.com</t>
+  </si>
+  <si>
+    <t>2001kumarharsh@gmail.com</t>
+  </si>
+  <si>
+    <t>Harsh Kumar</t>
   </si>
 </sst>
 </file>
@@ -486,6 +492,20 @@
         <v>4</v>
       </c>
     </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+    </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C6" s="2"/>
     </row>
@@ -502,8 +522,9 @@
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{2131B508-DA8F-4A27-BA2E-5B18E85D9CCA}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{F84ED4CC-95CF-4765-BFC2-35F5CEBB9CE7}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{4D26116C-C10F-4D0C-B76F-326FB1D7BC44}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId4"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
final changes and implemented the brevo
</commit_message>
<xml_diff>
--- a/all requirements/participants.xlsx
+++ b/all requirements/participants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HARDIK DHAWAN\OneDrive\Desktop\Minor-Project-Food-cupons-on-events-\all requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC942906-91A6-4B60-9167-33DF25315954}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA3947A1-E71E-4502-8298-4E0338C227CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="14">
   <si>
     <t>name</t>
   </si>
@@ -55,10 +55,13 @@
     <t>hardikdhawan446@gmail.com</t>
   </si>
   <si>
-    <t>2001kumarharsh@gmail.com</t>
-  </si>
-  <si>
-    <t>Harsh Kumar</t>
+    <t>Aaarv</t>
+  </si>
+  <si>
+    <t>team 2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ramesh </t>
   </si>
 </sst>
 </file>
@@ -497,12 +500,26 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
         <v>4</v>
       </c>
     </row>
@@ -522,9 +539,10 @@
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" xr:uid="{2131B508-DA8F-4A27-BA2E-5B18E85D9CCA}"/>
     <hyperlink ref="C3" r:id="rId2" xr:uid="{F84ED4CC-95CF-4765-BFC2-35F5CEBB9CE7}"/>
-    <hyperlink ref="C4" r:id="rId3" xr:uid="{4D26116C-C10F-4D0C-B76F-326FB1D7BC44}"/>
+    <hyperlink ref="C4" r:id="rId3" xr:uid="{05AE3C1A-934E-4E52-A019-3025898DC74C}"/>
+    <hyperlink ref="C5" r:id="rId4" xr:uid="{BE13AC28-82EE-4E68-872E-93FCCF13E167}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId4"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>